<commit_message>
Agregue codigo de oxxo, para lo cual tambien modifique los codigos de ejecucion para que puedan funcioanr con la generacion de varios Templare (tanto en Main como en Pruebas), tambien modifique El_Rosado para que corra correctamente. Por otro lado, tambien veerifique que todos los codigos que tenemos en el entorno de Prueba esten en el Main
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_farmatodo.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_farmatodo.xlsx
@@ -662,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -781,7 +781,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>15/10/2025</t>
+          <t>30/10/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1906,16 +1906,16 @@
     <row r="55">
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
         <is>
-          <t>PMP1289032</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E55" s="6" t="n">
-        <v>2.420000016689301</v>
+        <v>-4.769999992102385</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
@@ -1924,310 +1924,13 @@
       </c>
       <c r="G55" s="10" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>WOB</t>
         </is>
       </c>
       <c r="H55" s="6" t="n">
-        <v>2.420000016689301</v>
+        <v>-4.769999992102385</v>
       </c>
       <c r="I55" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="C56" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>PMP1289033</t>
-        </is>
-      </c>
-      <c r="E56" s="6" t="n">
-        <v>-0.1299999952316284</v>
-      </c>
-      <c r="F56" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="n">
-        <v>-0.1299999952316284</v>
-      </c>
-      <c r="I56" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="C57" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D57" s="10" t="inlineStr">
-        <is>
-          <t>PMP1289034</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="n">
-        <v>-0.3199999998323619</v>
-      </c>
-      <c r="F57" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G57" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="n">
-        <v>-0.3199999998323619</v>
-      </c>
-      <c r="I57" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="C58" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290566</t>
-        </is>
-      </c>
-      <c r="E58" s="6" t="n">
-        <v>-0.08000000007450581</v>
-      </c>
-      <c r="F58" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G58" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H58" s="6" t="n">
-        <v>-0.08000000007450581</v>
-      </c>
-      <c r="I58" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="C59" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290874</t>
-        </is>
-      </c>
-      <c r="E59" s="6" t="n">
-        <v>-0.9200000017881393</v>
-      </c>
-      <c r="F59" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G59" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H59" s="6" t="n">
-        <v>-0.9200000017881393</v>
-      </c>
-      <c r="I59" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290877</t>
-        </is>
-      </c>
-      <c r="E60" s="6" t="n">
-        <v>-0.1299999989569187</v>
-      </c>
-      <c r="F60" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G60" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H60" s="6" t="n">
-        <v>-0.1299999989569187</v>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290878</t>
-        </is>
-      </c>
-      <c r="E61" s="6" t="n">
-        <v>0.380000002682209</v>
-      </c>
-      <c r="F61" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G61" s="10" t="inlineStr">
-        <is>
-          <t>384</t>
-        </is>
-      </c>
-      <c r="H61" s="6" t="n">
-        <v>0.380000002682209</v>
-      </c>
-      <c r="I61" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="C62" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D62" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290879</t>
-        </is>
-      </c>
-      <c r="E62" s="6" t="n">
-        <v>0.3400000035762787</v>
-      </c>
-      <c r="F62" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G62" s="10" t="inlineStr">
-        <is>
-          <t>384</t>
-        </is>
-      </c>
-      <c r="H62" s="6" t="n">
-        <v>0.3400000035762787</v>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="C63" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290880</t>
-        </is>
-      </c>
-      <c r="E63" s="6" t="n">
-        <v>0.3999999999068677</v>
-      </c>
-      <c r="F63" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G63" s="10" t="inlineStr">
-        <is>
-          <t>384</t>
-        </is>
-      </c>
-      <c r="H63" s="6" t="n">
-        <v>0.3999999999068677</v>
-      </c>
-      <c r="I63" s="11" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="C64" s="10" t="inlineStr">
-        <is>
-          <t>Descuentos Clientes</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>PMP1290881</t>
-        </is>
-      </c>
-      <c r="E64" s="6" t="n">
-        <v>-6.730000019073486</v>
-      </c>
-      <c r="F64" s="10" t="inlineStr">
-        <is>
-          <t>MENORES VALORES</t>
-        </is>
-      </c>
-      <c r="G64" s="10" t="inlineStr">
-        <is>
-          <t>WOB</t>
-        </is>
-      </c>
-      <c r="H64" s="6" t="n">
-        <v>-6.730000019073486</v>
-      </c>
-      <c r="I64" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>

</xml_diff>

<commit_message>
Ajuste para que tome el importe del remittance en Farmatodo correctamente sin importar como venga el dato
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_farmatodo.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_farmatodo.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +55,13 @@
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -225,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -248,8 +255,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -261,13 +272,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -278,11 +289,17 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="15" fontId="7" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="15" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -649,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -659,8 +676,8 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -676,7 +693,7 @@
         </is>
       </c>
       <c r="H2" s="3" t="n">
-        <v>36385</v>
+        <v>1000170425</v>
       </c>
     </row>
     <row r="3"/>
@@ -705,7 +722,7 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>5565195.210000034</v>
+        <v>1941588376.66</v>
       </c>
     </row>
     <row r="7">
@@ -717,7 +734,7 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>5565195.210000034</v>
+        <v>1941588376.66</v>
       </c>
     </row>
     <row r="8">
@@ -764,11 +781,11 @@
     </row>
     <row r="12">
       <c r="C12" t="n">
-        <v>36385</v>
+        <v>1000170425</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>18/12/2025</t>
+          <t>29/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -777,7 +794,7 @@
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>5565195.210000034</v>
+        <v>1941588376.66</v>
       </c>
     </row>
     <row r="13"/>
@@ -830,16 +847,16 @@
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>PMP1310723</t>
+          <t>PMP1316267</t>
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>112253744.76</v>
+        <v>136849110.04</v>
       </c>
       <c r="F19" s="10" t="inlineStr"/>
       <c r="G19" s="10" t="inlineStr"/>
       <c r="H19" s="6" t="n">
-        <v>112253744.76</v>
+        <v>136849110.04</v>
       </c>
       <c r="I19" s="11" t="inlineStr"/>
     </row>
@@ -851,16 +868,16 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>PMP1310724</t>
+          <t>PMP1317481</t>
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>442526865.42</v>
+        <v>352537602.72</v>
       </c>
       <c r="F20" s="10" t="inlineStr"/>
       <c r="G20" s="10" t="inlineStr"/>
       <c r="H20" s="6" t="n">
-        <v>442526865.42</v>
+        <v>352537602.72</v>
       </c>
       <c r="I20" s="11" t="inlineStr"/>
     </row>
@@ -872,179 +889,123 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>PMP1311231</t>
+          <t>PMP1317482</t>
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>1862089</v>
+        <v>656318037.42</v>
       </c>
       <c r="F21" s="10" t="inlineStr"/>
       <c r="G21" s="10" t="inlineStr"/>
       <c r="H21" s="6" t="n">
-        <v>1862089</v>
+        <v>656318037.42</v>
       </c>
       <c r="I21" s="11" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Nota de Crédito</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>1200018001</t>
+          <t>PMP1317483</t>
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>-5565195</v>
-      </c>
-      <c r="F22" s="10" t="inlineStr">
-        <is>
-          <t>NRO</t>
-        </is>
-      </c>
+        <v>142583744.16</v>
+      </c>
+      <c r="F22" s="10" t="inlineStr"/>
       <c r="G22" s="10" t="inlineStr"/>
       <c r="H22" s="6" t="n">
-        <v>-5565195</v>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>favor del cliente sin aplicar por falta de soporte</t>
-        </is>
-      </c>
+        <v>142583744.16</v>
+      </c>
+      <c r="I22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>PMP1310723</t>
+          <t>PMP1317484</t>
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>-1886617.54</v>
-      </c>
-      <c r="F23" s="10" t="inlineStr">
-        <is>
-          <t>DPP</t>
-        </is>
-      </c>
-      <c r="G23" s="10" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
+        <v>44741671.96</v>
+      </c>
+      <c r="F23" s="10" t="inlineStr"/>
+      <c r="G23" s="10" t="inlineStr"/>
       <c r="H23" s="6" t="n">
-        <v>-1886617.54</v>
-      </c>
-      <c r="I23" s="11" t="inlineStr">
-        <is>
-          <t>DPP NC-PMP1310723</t>
-        </is>
-      </c>
+        <v>44741671.96</v>
+      </c>
+      <c r="I23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>PMP1310724</t>
+          <t>PMP1317485</t>
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>-7437426.31</v>
-      </c>
-      <c r="F24" s="10" t="inlineStr">
-        <is>
-          <t>DPP</t>
-        </is>
-      </c>
-      <c r="G24" s="10" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
+        <v>367332588.56</v>
+      </c>
+      <c r="F24" s="10" t="inlineStr"/>
+      <c r="G24" s="10" t="inlineStr"/>
       <c r="H24" s="6" t="n">
-        <v>-7437426.31</v>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>DPP NC-PMP1310724</t>
-        </is>
-      </c>
+        <v>367332588.56</v>
+      </c>
+      <c r="I24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>PMP1311231</t>
+          <t>PMP1318623</t>
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>-26792.64</v>
-      </c>
-      <c r="F25" s="10" t="inlineStr">
-        <is>
-          <t>DPP</t>
-        </is>
-      </c>
-      <c r="G25" s="10" t="inlineStr">
-        <is>
-          <t>206</t>
-        </is>
-      </c>
+        <v>187904609.44</v>
+      </c>
+      <c r="F25" s="10" t="inlineStr"/>
+      <c r="G25" s="10" t="inlineStr"/>
       <c r="H25" s="6" t="n">
-        <v>-26792.64</v>
-      </c>
-      <c r="I25" s="11" t="inlineStr">
-        <is>
-          <t>DPP NC-PMP1311231</t>
-        </is>
-      </c>
+        <v>187904609.44</v>
+      </c>
+      <c r="I25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Factura</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>PMP1310724</t>
+          <t>PMP1319923</t>
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>-656977.58</v>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>RECHAZOS</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>551</t>
-        </is>
-      </c>
+        <v>102414999.4</v>
+      </c>
+      <c r="F26" s="10" t="inlineStr"/>
+      <c r="G26" s="10" t="inlineStr"/>
       <c r="H26" s="6" t="n">
-        <v>-656977.58</v>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>RECHAZOS CNQPMP1310724</t>
-        </is>
-      </c>
+        <v>102414999.4</v>
+      </c>
+      <c r="I26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="C27" s="10" t="inlineStr">
@@ -1054,28 +1015,28 @@
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>DC04-555537</t>
+          <t>PMP1316267</t>
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>-149428373</v>
+        <v>-2299985.06</v>
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>DSCT PROMOCIONAL</t>
+          <t>DPP</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H27" s="6" t="n">
-        <v>-149428373</v>
+        <v>-2299985.06</v>
       </c>
       <c r="I27" s="11" t="inlineStr">
         <is>
-          <t>DSCT PROMOCIONAL NC-DC04-555537</t>
+          <t>DPP NC-PMP1316267</t>
         </is>
       </c>
     </row>
@@ -1087,28 +1048,28 @@
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>FV-XKZV33203</t>
+          <t>PMP1317481</t>
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>-96522911.92</v>
+        <v>-5925001.73</v>
       </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>DPP</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H28" s="6" t="n">
-        <v>-96522911.92</v>
+        <v>-5925001.73</v>
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR FV-XKZV33203</t>
+          <t>DPP NC-PMP1317481</t>
         </is>
       </c>
     </row>
@@ -1120,28 +1081,28 @@
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>FV-XKZV33397</t>
+          <t>PMP1317482</t>
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>-602319.64</v>
+        <v>-11030555.21</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>DPP</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H29" s="6" t="n">
-        <v>-602319.64</v>
+        <v>-11030555.21</v>
       </c>
       <c r="I29" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR FV-XKZV33397</t>
+          <t>DPP NC-PMP1317482</t>
         </is>
       </c>
     </row>
@@ -1153,28 +1114,28 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>FV-XKZV33514</t>
+          <t>PMP1317483</t>
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>-294516083.33</v>
+        <v>-2396365.48</v>
       </c>
       <c r="F30" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>DPP</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H30" s="6" t="n">
-        <v>-294516083.33</v>
+        <v>-2396365.48</v>
       </c>
       <c r="I30" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR FV-XKZV33514</t>
+          <t>DPP NC-PMP1317483</t>
         </is>
       </c>
     </row>
@@ -1186,26 +1147,554 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
+          <t>PMP1317484</t>
+        </is>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>-751960.86</v>
+      </c>
+      <c r="F31" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>-751960.86</v>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>DPP NC-PMP1317484</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317485</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>-6173656.93</v>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>-6173656.93</v>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>DPP NC-PMP1317485</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>PMP1318623</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>-3158060.67</v>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>-3158060.67</v>
+      </c>
+      <c r="I33" s="11" t="inlineStr">
+        <is>
+          <t>DPP NC-PMP1318623</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>PMP1319923</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>-1721260.45</v>
+      </c>
+      <c r="F34" s="10" t="inlineStr">
+        <is>
+          <t>DPP</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>-1721260.45</v>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>DPP NC-PMP1319923</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>NC100349505</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>-3880114</v>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t>DSCT AVERIAS</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>522</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>-3880114</v>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>DSCT AVERIAS NC100349505</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="C36" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>PMP1316267</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>-390931.18</v>
+      </c>
+      <c r="F36" s="10" t="inlineStr">
+        <is>
+          <t>RECHAZOS</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>-390931.18</v>
+      </c>
+      <c r="I36" s="11" t="inlineStr">
+        <is>
+          <t>RECHAZOS CNQPMP1316267</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="C37" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317481</t>
+        </is>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>-124626.32</v>
+      </c>
+      <c r="F37" s="10" t="inlineStr">
+        <is>
+          <t>RECHAZOS</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>-124626.32</v>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>RECHAZOS CNQPMP1317481</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317482</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>-3256197</v>
+      </c>
+      <c r="F38" s="10" t="inlineStr">
+        <is>
+          <t>RECHAZOS</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>-3256197</v>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>RECHAZOS CNQPMP1317482</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317485</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>-7985268.9</v>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>RECHAZOS</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>551</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>-7985268.9</v>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>RECHAZOS CNQPMP1317485</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>PMP1316267</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>1.080000013113022</v>
+      </c>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
           <t>MENORES VALORES</t>
         </is>
       </c>
-      <c r="E31" s="6" t="n">
-        <v>-2.009999994654208</v>
-      </c>
-      <c r="F31" s="10" t="inlineStr">
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>1.080000013113022</v>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>
       </c>
-      <c r="G31" s="10" t="inlineStr">
-        <is>
-          <t>CSR</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="n">
-        <v>-2.009999994654208</v>
-      </c>
-      <c r="I31" s="11" t="inlineStr">
+    </row>
+    <row r="41">
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317481</t>
+        </is>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>0.4799999594688416</v>
+      </c>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>0.4799999594688416</v>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317483</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>2.090000003576279</v>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>2.090000003576279</v>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="C43" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>PMP1318623</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>0.3499999940395355</v>
+      </c>
+      <c r="F43" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G43" s="10" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>0.3499999940395355</v>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317482</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>-2.519999980926514</v>
+      </c>
+      <c r="F44" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>-2.519999980926514</v>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="C45" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D45" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317484</t>
+        </is>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>-0.8400000035762787</v>
+      </c>
+      <c r="F45" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G45" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>-0.8400000035762787</v>
+      </c>
+      <c r="I45" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D46" s="10" t="inlineStr">
+        <is>
+          <t>PMP1317485</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>-1.149999976158142</v>
+      </c>
+      <c r="F46" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G46" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>-1.149999976158142</v>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>Descuentos Clientes</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>PMP1319923</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>-2.740000009536743</v>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>MENORES VALORES</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="inlineStr">
+        <is>
+          <t>WOB</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>-2.740000009536743</v>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
         <is>
           <t>MENORES VALORES</t>
         </is>
@@ -1222,27 +1711,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11.6640625" customWidth="1" min="1" max="1"/>
-    <col width="9.4140625" customWidth="1" min="2" max="2"/>
-    <col width="12.25" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13.33203125" customWidth="1" min="5" max="5"/>
-    <col width="17.08203125" customWidth="1" min="6" max="6"/>
-    <col width="14.1640625" customWidth="1" min="7" max="7"/>
-    <col width="37" customWidth="1" min="8" max="8"/>
-    <col width="22.75" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="14.33203125" customWidth="1" min="11" max="11"/>
-    <col width="20.75" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="14.33203125" customWidth="1" min="14" max="14"/>
-    <col width="15.58203125" customWidth="1" min="15" max="15"/>
+    <col width="14.83203125" customWidth="1" min="4" max="4"/>
+    <col width="31.5" customWidth="1" min="8" max="8"/>
+    <col width="14.1640625" customWidth="1" min="9" max="9"/>
+    <col width="16.6640625" customWidth="1" min="10" max="10"/>
+    <col width="18.6640625" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1">
+    <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>FARMATODO COLOMBIA, S.A.</t>
@@ -1250,7 +1729,7 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Nit  830129327-1</t>
@@ -1265,7 +1744,7 @@
       </c>
     </row>
     <row r="5"/>
-    <row r="6" ht="16.65" customHeight="1">
+    <row r="6" ht="34" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Banco</t>
@@ -1302,24 +1781,22 @@
       <c r="N6" s="17" t="n"/>
       <c r="O6" s="18" t="n"/>
     </row>
-    <row r="7" ht="15.65" customHeight="1">
+    <row r="7" ht="17" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
         <is>
-          <t>PROSEGUR</t>
+          <t>BANCOLOMBIA</t>
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>36385</v>
+        <v>1000170425</v>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>‭09-DIC-2025‬</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>5.565.195,21</t>
-        </is>
+          <t>‭26-DIC-2025‬</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>1941588376.66</v>
       </c>
       <c r="E7" s="20" t="inlineStr">
         <is>
@@ -1377,7 +1854,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15.65" customHeight="1">
+    <row r="8" ht="17" customHeight="1">
       <c r="A8" s="23" t="n"/>
       <c r="B8" s="23" t="n"/>
       <c r="C8" s="23" t="n"/>
@@ -1398,7 +1875,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15.65" customHeight="1">
+    <row r="9" ht="34" customHeight="1">
       <c r="A9" s="23" t="n"/>
       <c r="B9" s="23" t="n"/>
       <c r="C9" s="23" t="n"/>
@@ -1406,56 +1883,40 @@
       <c r="E9" s="23" t="n"/>
       <c r="F9" s="20" t="inlineStr">
         <is>
-          <t>‭FV-XKZV33203‬</t>
-        </is>
-      </c>
-      <c r="G9" s="20" t="inlineStr">
-        <is>
-          <t>03-DIC-2025</t>
-        </is>
-      </c>
-      <c r="H9" s="19" t="inlineStr">
-        <is>
-          <t>Acuerdo Fijo Mensual 01 2.3%  - MASIVOS/MISCELANEOS Logístico</t>
-        </is>
-      </c>
-      <c r="I9" s="21" t="inlineStr">
-        <is>
-          <t>-96.522.911,92</t>
-        </is>
-      </c>
-      <c r="J9" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K9" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L9" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M9" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N9" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O9" s="21" t="inlineStr">
-        <is>
-          <t>-96.522.911,92</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15.65" customHeight="1">
+          <t>‭PMP1317484‬</t>
+        </is>
+      </c>
+      <c r="G9" s="26" t="n">
+        <v>45994</v>
+      </c>
+      <c r="H9" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015315 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I9" s="28" t="n">
+        <v>37598042.96</v>
+      </c>
+      <c r="J9" s="28" t="n">
+        <v>7143628.16</v>
+      </c>
+      <c r="K9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="28" t="n">
+        <v>44741671.12</v>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
       <c r="A10" s="23" t="n"/>
       <c r="B10" s="23" t="n"/>
       <c r="C10" s="23" t="n"/>
@@ -1463,56 +1924,40 @@
       <c r="E10" s="23" t="n"/>
       <c r="F10" s="20" t="inlineStr">
         <is>
-          <t>‭FV-XKZV33397‬</t>
-        </is>
-      </c>
-      <c r="G10" s="20" t="inlineStr">
-        <is>
-          <t>03-DIC-2025</t>
-        </is>
-      </c>
-      <c r="H10" s="19" t="inlineStr">
-        <is>
-          <t>Acuerdo Fijo Mensual 01 7%  - MASIVOS/MISCELANEOS Exhibiciones Adicionales</t>
-        </is>
-      </c>
-      <c r="I10" s="21" t="inlineStr">
-        <is>
-          <t>-602.319,64</t>
-        </is>
-      </c>
-      <c r="J10" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K10" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L10" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M10" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N10" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O10" s="21" t="inlineStr">
-        <is>
-          <t>-602.319,64</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15.65" customHeight="1">
+          <t>‭PMP1317485‬</t>
+        </is>
+      </c>
+      <c r="G10" s="26" t="n">
+        <v>45994</v>
+      </c>
+      <c r="H10" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015315 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I10" s="28" t="n">
+        <v>308682846.56</v>
+      </c>
+      <c r="J10" s="28" t="n">
+        <v>58649740.85</v>
+      </c>
+      <c r="K10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="28" t="n">
+        <v>367332587.41</v>
+      </c>
+    </row>
+    <row r="11" ht="51" customHeight="1">
       <c r="A11" s="23" t="n"/>
       <c r="B11" s="23" t="n"/>
       <c r="C11" s="23" t="n"/>
@@ -1520,56 +1965,40 @@
       <c r="E11" s="23" t="n"/>
       <c r="F11" s="20" t="inlineStr">
         <is>
-          <t>‭FV-XKZV33514‬</t>
-        </is>
-      </c>
-      <c r="G11" s="20" t="inlineStr">
-        <is>
-          <t>03-DIC-2025</t>
-        </is>
-      </c>
-      <c r="H11" s="19" t="inlineStr">
-        <is>
-          <t>EXHIBICIONES ADICIONALES NOVIEMBRE 2025</t>
-        </is>
-      </c>
-      <c r="I11" s="21" t="inlineStr">
-        <is>
-          <t>-294.516.083,33</t>
-        </is>
-      </c>
-      <c r="J11" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K11" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L11" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M11" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N11" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O11" s="21" t="inlineStr">
-        <is>
-          <t>-294.516.083,33</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15.65" customHeight="1">
+          <t>‭NC-PMP1317484‬</t>
+        </is>
+      </c>
+      <c r="G11" s="26" t="n">
+        <v>45994</v>
+      </c>
+      <c r="H11" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015315 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="28" t="n">
+        <v>-751960.86</v>
+      </c>
+      <c r="N11" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="28" t="n">
+        <v>-751960.86</v>
+      </c>
+    </row>
+    <row r="12" ht="51" customHeight="1">
       <c r="A12" s="23" t="n"/>
       <c r="B12" s="23" t="n"/>
       <c r="C12" s="23" t="n"/>
@@ -1577,56 +2006,40 @@
       <c r="E12" s="23" t="n"/>
       <c r="F12" s="20" t="inlineStr">
         <is>
-          <t>‭NC-DC04-555537‬</t>
-        </is>
-      </c>
-      <c r="G12" s="20" t="inlineStr">
-        <is>
-          <t>03-DIC-2025</t>
-        </is>
-      </c>
-      <c r="H12" s="19" t="inlineStr">
-        <is>
-          <t>Miscelaneos : Liquidaciones Ventas Pos-Folleto Quincenal 24 Octubre al 6 Noviembre  -Belleza y CP</t>
-        </is>
-      </c>
-      <c r="I12" s="21" t="inlineStr">
-        <is>
-          <t>-149.428.373,00</t>
-        </is>
-      </c>
-      <c r="J12" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K12" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L12" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M12" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N12" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O12" s="21" t="inlineStr">
-        <is>
-          <t>-149.428.373,00</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15.65" customHeight="1">
+          <t>‭NC-PMP1317485‬</t>
+        </is>
+      </c>
+      <c r="G12" s="26" t="n">
+        <v>45994</v>
+      </c>
+      <c r="H12" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015315 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="28" t="n">
+        <v>-6173656.93</v>
+      </c>
+      <c r="N12" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="28" t="n">
+        <v>-6173656.93</v>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
       <c r="A13" s="23" t="n"/>
       <c r="B13" s="23" t="n"/>
       <c r="C13" s="23" t="n"/>
@@ -1634,56 +2047,40 @@
       <c r="E13" s="23" t="n"/>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>‭CNQPMP1310724‬</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>05-DIC-2025</t>
-        </is>
-      </c>
-      <c r="H13" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013732 UNILEVER ANDINA COLOMBIA LTDA</t>
-        </is>
-      </c>
-      <c r="I13" s="21" t="inlineStr">
-        <is>
-          <t>-552.082,00</t>
-        </is>
-      </c>
-      <c r="J13" s="21" t="inlineStr">
-        <is>
-          <t>-104.895,58</t>
-        </is>
-      </c>
-      <c r="K13" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L13" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M13" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N13" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O13" s="21" t="inlineStr">
-        <is>
-          <t>-656.977,58</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15.65" customHeight="1">
+          <t>‭PMP1317481‬</t>
+        </is>
+      </c>
+      <c r="G13" s="26" t="n">
+        <v>45994</v>
+      </c>
+      <c r="H13" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I13" s="28" t="n">
+        <v>296250086.72</v>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>56287516.48</v>
+      </c>
+      <c r="K13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="28" t="n">
+        <v>352537603.2</v>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="23" t="n"/>
       <c r="B14" s="23" t="n"/>
       <c r="C14" s="23" t="n"/>
@@ -1691,54 +2088,40 @@
       <c r="E14" s="23" t="n"/>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>‭PMP1310724‬</t>
+          <t>‭PMP1317482‬</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>45976</v>
-      </c>
-      <c r="H14" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013732 UNILEVER ANDINA COLOMBIA LTDA</t>
-        </is>
-      </c>
-      <c r="I14" s="21" t="inlineStr">
-        <is>
-          <t>371.871.315,42</t>
-        </is>
-      </c>
-      <c r="J14" s="21" t="inlineStr">
-        <is>
-          <t>70.655.549,93</t>
-        </is>
-      </c>
-      <c r="K14" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L14" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M14" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N14" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O14" s="21" t="inlineStr">
-        <is>
-          <t>442.526.865,35</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15.65" customHeight="1">
+        <v>45994</v>
+      </c>
+      <c r="H14" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I14" s="28" t="n">
+        <v>551527760.42</v>
+      </c>
+      <c r="J14" s="28" t="n">
+        <v>104790274.48</v>
+      </c>
+      <c r="K14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="28" t="n">
+        <v>656318034.9</v>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
       <c r="A15" s="23" t="n"/>
       <c r="B15" s="23" t="n"/>
       <c r="C15" s="23" t="n"/>
@@ -1746,54 +2129,40 @@
       <c r="E15" s="23" t="n"/>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>‭NC-PMP1310723‬</t>
+          <t>‭PMP1317483‬</t>
         </is>
       </c>
       <c r="G15" s="26" t="n">
-        <v>45976</v>
-      </c>
-      <c r="H15" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013732 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
-        </is>
-      </c>
-      <c r="I15" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="J15" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K15" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L15" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M15" s="21" t="inlineStr">
-        <is>
-          <t>-1.886.617,54</t>
-        </is>
-      </c>
-      <c r="N15" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O15" s="21" t="inlineStr">
-        <is>
-          <t>-1.886.617,54</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15.65" customHeight="1">
+        <v>45994</v>
+      </c>
+      <c r="H15" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I15" s="28" t="n">
+        <v>119818274.16</v>
+      </c>
+      <c r="J15" s="28" t="n">
+        <v>22765472.09</v>
+      </c>
+      <c r="K15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="28" t="n">
+        <v>142583746.25</v>
+      </c>
+    </row>
+    <row r="16" ht="51" customHeight="1">
       <c r="A16" s="23" t="n"/>
       <c r="B16" s="23" t="n"/>
       <c r="C16" s="23" t="n"/>
@@ -1801,54 +2170,40 @@
       <c r="E16" s="23" t="n"/>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>‭NC-PMP1310724‬</t>
+          <t>‭NC-PMP1317481‬</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>45976</v>
-      </c>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013732 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
-        </is>
-      </c>
-      <c r="I16" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="J16" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K16" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L16" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M16" s="21" t="inlineStr">
-        <is>
-          <t>-7.437.426,31</t>
-        </is>
-      </c>
-      <c r="N16" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O16" s="21" t="inlineStr">
-        <is>
-          <t>-7.437.426,31</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15.65" customHeight="1">
+        <v>45994</v>
+      </c>
+      <c r="H16" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="28" t="n">
+        <v>-5925001.73</v>
+      </c>
+      <c r="N16" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="28" t="n">
+        <v>-5925001.73</v>
+      </c>
+    </row>
+    <row r="17" ht="51" customHeight="1">
       <c r="A17" s="23" t="n"/>
       <c r="B17" s="23" t="n"/>
       <c r="C17" s="23" t="n"/>
@@ -1856,54 +2211,40 @@
       <c r="E17" s="23" t="n"/>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>‭PMP1310723‬</t>
+          <t>‭NC-PMP1317482‬</t>
         </is>
       </c>
       <c r="G17" s="26" t="n">
-        <v>45976</v>
-      </c>
-      <c r="H17" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013732 UNILEVER ANDINA COLOMBIA LTDA</t>
-        </is>
-      </c>
-      <c r="I17" s="21" t="inlineStr">
-        <is>
-          <t>94.330.876,76</t>
-        </is>
-      </c>
-      <c r="J17" s="21" t="inlineStr">
-        <is>
-          <t>17.922.866,58</t>
-        </is>
-      </c>
-      <c r="K17" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L17" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M17" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N17" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O17" s="21" t="inlineStr">
-        <is>
-          <t>112.253.743,34</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15.65" customHeight="1">
+        <v>45994</v>
+      </c>
+      <c r="H17" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="28" t="n">
+        <v>-11030555.21</v>
+      </c>
+      <c r="N17" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="28" t="n">
+        <v>-11030555.21</v>
+      </c>
+    </row>
+    <row r="18" ht="51" customHeight="1">
       <c r="A18" s="23" t="n"/>
       <c r="B18" s="23" t="n"/>
       <c r="C18" s="23" t="n"/>
@@ -1911,135 +2252,506 @@
       <c r="E18" s="23" t="n"/>
       <c r="F18" s="20" t="inlineStr">
         <is>
-          <t>‭NC-PMP1311231‬</t>
+          <t>‭NC-PMP1317483‬</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>45977</v>
-      </c>
-      <c r="H18" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013771 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
-        </is>
-      </c>
-      <c r="I18" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="J18" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="K18" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L18" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M18" s="21" t="inlineStr">
-        <is>
-          <t>-26.792,64</t>
-        </is>
-      </c>
-      <c r="N18" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O18" s="21" t="inlineStr">
-        <is>
-          <t>-26.792,64</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15.65" customHeight="1">
-      <c r="A19" s="24" t="n"/>
-      <c r="B19" s="24" t="n"/>
-      <c r="C19" s="24" t="n"/>
-      <c r="D19" s="24" t="n"/>
-      <c r="E19" s="24" t="n"/>
+        <v>45994</v>
+      </c>
+      <c r="H18" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="28" t="n">
+        <v>-2396365.48</v>
+      </c>
+      <c r="N18" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="28" t="n">
+        <v>-2396365.48</v>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="23" t="n"/>
+      <c r="D19" s="23" t="n"/>
+      <c r="E19" s="23" t="n"/>
       <c r="F19" s="20" t="inlineStr">
         <is>
-          <t>‭PMP1311231‬</t>
+          <t>‭PMP1318623‬</t>
         </is>
       </c>
       <c r="G19" s="26" t="n">
-        <v>45977</v>
-      </c>
-      <c r="H19" s="19" t="inlineStr">
-        <is>
-          <t>OC:14013771 UNILEVER ANDINA COLOMBIA LTDA</t>
-        </is>
-      </c>
-      <c r="I19" s="21" t="inlineStr">
-        <is>
-          <t>1.607.558,40</t>
-        </is>
-      </c>
-      <c r="J19" s="21" t="inlineStr">
-        <is>
-          <t>254.530,08</t>
-        </is>
-      </c>
-      <c r="K19" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="L19" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="M19" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="N19" s="21" t="inlineStr">
-        <is>
-          <t>0,00</t>
-        </is>
-      </c>
-      <c r="O19" s="21" t="inlineStr">
-        <is>
-          <t>1.862.088,48</t>
-        </is>
-      </c>
-    </row>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23" ht="15.5" customHeight="1">
-      <c r="A23" s="27" t="inlineStr">
-        <is>
-          <t>                     </t>
-        </is>
+        <v>45996</v>
+      </c>
+      <c r="H19" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015742 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I19" s="28" t="n">
+        <v>157903033.44</v>
+      </c>
+      <c r="J19" s="28" t="n">
+        <v>30001576.35</v>
+      </c>
+      <c r="K19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="28" t="n">
+        <v>187904609.79</v>
+      </c>
+    </row>
+    <row r="20" ht="51" customHeight="1">
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="23" t="n"/>
+      <c r="D20" s="23" t="n"/>
+      <c r="E20" s="23" t="n"/>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>‭NC-PMP1318623‬</t>
+        </is>
+      </c>
+      <c r="G20" s="26" t="n">
+        <v>45996</v>
+      </c>
+      <c r="H20" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015742 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="28" t="n">
+        <v>-3158060.67</v>
+      </c>
+      <c r="N20" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="28" t="n">
+        <v>-3158060.67</v>
+      </c>
+    </row>
+    <row r="21" ht="51" customHeight="1">
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="23" t="n"/>
+      <c r="D21" s="23" t="n"/>
+      <c r="E21" s="23" t="n"/>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>‭NC-PMP1319923‬</t>
+        </is>
+      </c>
+      <c r="G21" s="26" t="n">
+        <v>46000</v>
+      </c>
+      <c r="H21" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015935 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="28" t="n">
+        <v>-1721260.45</v>
+      </c>
+      <c r="N21" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="28" t="n">
+        <v>-1721260.45</v>
+      </c>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="23" t="n"/>
+      <c r="D22" s="23" t="n"/>
+      <c r="E22" s="23" t="n"/>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>‭PMP1319923‬</t>
+        </is>
+      </c>
+      <c r="G22" s="26" t="n">
+        <v>46000</v>
+      </c>
+      <c r="H22" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015935 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I22" s="28" t="n">
+        <v>86063022.40000001</v>
+      </c>
+      <c r="J22" s="28" t="n">
+        <v>16351974.26</v>
+      </c>
+      <c r="K22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="28" t="n">
+        <v>102414996.66</v>
+      </c>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="23" t="n"/>
+      <c r="B23" s="23" t="n"/>
+      <c r="C23" s="23" t="n"/>
+      <c r="D23" s="23" t="n"/>
+      <c r="E23" s="23" t="n"/>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>‭NC100349505‬</t>
+        </is>
+      </c>
+      <c r="G23" s="26" t="n">
+        <v>46014</v>
+      </c>
+      <c r="H23" s="27" t="inlineStr">
+        <is>
+          <t>NOTAS DE CREDITO POR DEVOLUCION 100349505</t>
+        </is>
+      </c>
+      <c r="I23" s="28" t="n">
+        <v>-3260600</v>
+      </c>
+      <c r="J23" s="28" t="n">
+        <v>-619514</v>
+      </c>
+      <c r="K23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="28" t="n">
+        <v>-3880114</v>
+      </c>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="23" t="n"/>
+      <c r="B24" s="23" t="n"/>
+      <c r="C24" s="23" t="n"/>
+      <c r="D24" s="23" t="n"/>
+      <c r="E24" s="23" t="n"/>
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>‭CNQPMP1316267‬</t>
+        </is>
+      </c>
+      <c r="G24" s="26" t="n">
+        <v>46014</v>
+      </c>
+      <c r="H24" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015148 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I24" s="28" t="n">
+        <v>-328513.6</v>
+      </c>
+      <c r="J24" s="28" t="n">
+        <v>-62417.58</v>
+      </c>
+      <c r="K24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="28" t="n">
+        <v>-390931.18</v>
+      </c>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="23" t="n"/>
+      <c r="B25" s="23" t="n"/>
+      <c r="C25" s="23" t="n"/>
+      <c r="D25" s="23" t="n"/>
+      <c r="E25" s="23" t="n"/>
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>‭CNQPMP1317485‬</t>
+        </is>
+      </c>
+      <c r="G25" s="26" t="n">
+        <v>46017</v>
+      </c>
+      <c r="H25" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015315 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I25" s="28" t="n">
+        <v>-6710310</v>
+      </c>
+      <c r="J25" s="28" t="n">
+        <v>-1274958.9</v>
+      </c>
+      <c r="K25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="28" t="n">
+        <v>-7985268.9</v>
+      </c>
+    </row>
+    <row r="26" ht="34" customHeight="1">
+      <c r="A26" s="23" t="n"/>
+      <c r="B26" s="23" t="n"/>
+      <c r="C26" s="23" t="n"/>
+      <c r="D26" s="23" t="n"/>
+      <c r="E26" s="23" t="n"/>
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>‭CNQPMP1317481‬</t>
+        </is>
+      </c>
+      <c r="G26" s="26" t="n">
+        <v>46017</v>
+      </c>
+      <c r="H26" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I26" s="28" t="n">
+        <v>-104728</v>
+      </c>
+      <c r="J26" s="28" t="n">
+        <v>-19898.32</v>
+      </c>
+      <c r="K26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="28" t="n">
+        <v>-124626.32</v>
+      </c>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="23" t="n"/>
+      <c r="B27" s="23" t="n"/>
+      <c r="C27" s="23" t="n"/>
+      <c r="D27" s="23" t="n"/>
+      <c r="E27" s="23" t="n"/>
+      <c r="F27" s="20" t="inlineStr">
+        <is>
+          <t>‭CNQPMP1317482‬</t>
+        </is>
+      </c>
+      <c r="G27" s="26" t="n">
+        <v>46017</v>
+      </c>
+      <c r="H27" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015435 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I27" s="28" t="n">
+        <v>-2736300</v>
+      </c>
+      <c r="J27" s="28" t="n">
+        <v>-519897</v>
+      </c>
+      <c r="K27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="28" t="n">
+        <v>-3256197</v>
+      </c>
+    </row>
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="23" t="n"/>
+      <c r="B28" s="23" t="n"/>
+      <c r="C28" s="23" t="n"/>
+      <c r="D28" s="23" t="n"/>
+      <c r="E28" s="23" t="n"/>
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>‭PMP1316267‬</t>
+        </is>
+      </c>
+      <c r="G28" s="26" t="n">
+        <v>45989</v>
+      </c>
+      <c r="H28" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015148 UNILEVER ANDINA COLOMBIA LTDA</t>
+        </is>
+      </c>
+      <c r="I28" s="28" t="n">
+        <v>114999253.04</v>
+      </c>
+      <c r="J28" s="28" t="n">
+        <v>21849858.08</v>
+      </c>
+      <c r="K28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="28" t="n">
+        <v>136849111.12</v>
+      </c>
+    </row>
+    <row r="29" ht="51" customHeight="1">
+      <c r="A29" s="24" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="20" t="inlineStr">
+        <is>
+          <t>‭NC-PMP1316267‬</t>
+        </is>
+      </c>
+      <c r="G29" s="26" t="n">
+        <v>45989</v>
+      </c>
+      <c r="H29" s="27" t="inlineStr">
+        <is>
+          <t>OC:14015148 UNILEVER ANDINA COLOMBIA LTDA (DPP)</t>
+        </is>
+      </c>
+      <c r="I29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="28" t="n">
+        <v>-2299985.06</v>
+      </c>
+      <c r="N29" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="28" t="n">
+        <v>-2299985.06</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
-    <mergeCell ref="M7:M8"/>
-    <mergeCell ref="C7:C19"/>
-    <mergeCell ref="A7:A19"/>
-    <mergeCell ref="B7:B19"/>
-    <mergeCell ref="A23:O23"/>
-    <mergeCell ref="D7:D19"/>
-    <mergeCell ref="E7:E19"/>
+  <mergeCells count="15">
+    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="C7:C29"/>
+    <mergeCell ref="A7:A29"/>
+    <mergeCell ref="D7:D29"/>
+    <mergeCell ref="B7:B29"/>
+    <mergeCell ref="E7:E29"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="H7:H8"/>
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="L7:L8"/>
-    <mergeCell ref="G7:G8"/>
-    <mergeCell ref="H7:H8"/>
-    <mergeCell ref="N7:N8"/>
+    <mergeCell ref="J7:J8"/>
     <mergeCell ref="I7:I8"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="M7:M8"/>
     <mergeCell ref="F6:O6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>